<commit_message>
Add Group 3 Week 4 project document
</commit_message>
<xml_diff>
--- a/Capstone_Project/00_Project_Administration/Group-3_Project_Attendance_Register.xlsx
+++ b/Capstone_Project/00_Project_Administration/Group-3_Project_Attendance_Register.xlsx
@@ -17,9 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="ddd dd mmm yyyy"/>
     <numFmt numFmtId="165" formatCode="hh:mm"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -213,6 +214,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -238,6 +242,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -263,6 +270,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -288,6 +298,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -313,6 +326,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -332,6 +348,59 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="476250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1038,26 +1107,78 @@
       </c>
       <c r="I12" s="2" t="n"/>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
+    <row r="13" ht="44" customHeight="1" s="4">
+      <c r="A13" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>20230260</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Thomas du Plessis</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Group 3</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>0.5284722222222222</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>0.6118055555555556</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Task 7 Lecturer slots page</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Lecturer slots page (commit c2ecca1 and pull request #6 merged at 14:56)</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="n"/>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
+    <row r="14" ht="44" customHeight="1" s="4">
+      <c r="A14" s="7" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>20230257</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Willem Gerber</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Group 3</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>0.6118055555555556</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>0.6222222222222222</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Review Thomas pull request</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Reviewed and merged pull request #6</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="n"/>
     </row>
     <row r="15">

</xml_diff>